<commit_message>
correção para a emissão da NFSe da prefeitura de Campinas.
</commit_message>
<xml_diff>
--- a/examples/edm_teste_campinas_resultado.xlsx
+++ b/examples/edm_teste_campinas_resultado.xlsx
@@ -648,7 +648,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>12750</v>
+        <v>12752</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>46174</v>
@@ -724,7 +724,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>S</t>
+          <t>N</t>
         </is>
       </c>
       <c r="V2" t="n">
@@ -745,7 +745,7 @@
       <c r="AF2" t="inlineStr"/>
       <c r="AG2" t="inlineStr">
         <is>
-          <t>{http://nfse.abrasf.org.br}RecepcionarLoteRpsSincrono() got an unexpected keyword argument 'nfseCabecMsg'. Signature: `EnviarLoteRpsSincronoEnvio: {LoteRps: {http://www.abrasf.org.br/nfse.xsd}tcLoteRps, Signature: {http://www.w3.org/2000/09/xmldsig#}SignatureType}`</t>
+          <t xml:space="preserve">Webservice retornou erro(s): L999: </t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
emissão em homologação concluído com sucesso.
</commit_message>
<xml_diff>
--- a/examples/edm_teste_campinas_resultado.xlsx
+++ b/examples/edm_teste_campinas_resultado.xlsx
@@ -26,6 +26,7 @@
     </font>
     <font>
       <name val="Calibri"/>
+      <family val="2"/>
       <b val="1"/>
       <color rgb="FFFFFFFF"/>
       <sz val="9"/>
@@ -58,7 +59,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00FFC7CE"/>
+        <fgColor rgb="00C6EFCE"/>
       </patternFill>
     </fill>
   </fills>
@@ -592,7 +593,7 @@
       </c>
       <c r="W1" s="2" t="inlineStr">
         <is>
-          <t>Código CNAE</t>
+          <t>Código CNAE (7 ou 9 dígitos)</t>
         </is>
       </c>
       <c r="X1" s="3" t="inlineStr">
@@ -730,24 +731,26 @@
       <c r="V2" t="n">
         <v>1</v>
       </c>
-      <c r="W2" t="inlineStr">
-        <is>
-          <t>6920601</t>
-        </is>
+      <c r="W2" t="n">
+        <v>692060100</v>
       </c>
       <c r="AC2" s="6" t="inlineStr">
         <is>
-          <t>ERRO</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr"/>
-      <c r="AE2" t="inlineStr"/>
+          <t>EMITIDA</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr">
+        <is>
+          <t>18698</t>
+        </is>
+      </c>
+      <c r="AE2" t="inlineStr">
+        <is>
+          <t>ekIo2vVSB</t>
+        </is>
+      </c>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr">
-        <is>
-          <t xml:space="preserve">Webservice retornou erro(s): L999: </t>
-        </is>
-      </c>
+      <c r="AG2" t="inlineStr"/>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>

<commit_message>
implementação da consulta de número de RPS e correção da implementação em produção. alterado onde ficar a informação de SIMPLES NACIONAL.
</commit_message>
<xml_diff>
--- a/examples/edm_teste_campinas_resultado.xlsx
+++ b/examples/edm_teste_campinas_resultado.xlsx
@@ -59,7 +59,7 @@
     </fill>
     <fill>
       <patternFill patternType="solid">
-        <fgColor rgb="00C6EFCE"/>
+        <fgColor rgb="00FFC7CE"/>
       </patternFill>
     </fill>
   </fills>
@@ -649,7 +649,7 @@
     </row>
     <row r="2">
       <c r="A2" t="n">
-        <v>12752</v>
+        <v>1</v>
       </c>
       <c r="B2" s="4" t="n">
         <v>46174</v>
@@ -725,7 +725,7 @@
       </c>
       <c r="U2" t="inlineStr">
         <is>
-          <t>N</t>
+          <t>S</t>
         </is>
       </c>
       <c r="V2" t="n">
@@ -736,21 +736,17 @@
       </c>
       <c r="AC2" s="6" t="inlineStr">
         <is>
-          <t>EMITIDA</t>
-        </is>
-      </c>
-      <c r="AD2" t="inlineStr">
-        <is>
-          <t>18698</t>
-        </is>
-      </c>
-      <c r="AE2" t="inlineStr">
-        <is>
-          <t>ekIo2vVSB</t>
-        </is>
-      </c>
+          <t>ERRO</t>
+        </is>
+      </c>
+      <c r="AD2" t="inlineStr"/>
+      <c r="AE2" t="inlineStr"/>
       <c r="AF2" t="inlineStr"/>
-      <c r="AG2" t="inlineStr"/>
+      <c r="AG2" t="inlineStr">
+        <is>
+          <t>Webservice retornou erro(s): E10: Tipo: 1 Série: 1 Número: 1 já informado anteriormente</t>
+        </is>
+      </c>
     </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>

</xml_diff>